<commit_message>
New Month Start Day 16
</commit_message>
<xml_diff>
--- a/12620583.xlsx
+++ b/12620583.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VITHOBA_12620583\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C73FDBA0-D00D-444A-9F5B-186199E8F02A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC54A7D8-1C99-4298-9BFA-9862C6E0CF20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -202,9 +202,6 @@
     <t>MCA / D1P2536</t>
   </si>
   <si>
-    <t>August</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Sleep (min)</t>
   </si>
   <si>
@@ -269,6 +266,12 @@
   </si>
   <si>
     <t>starting study for CA .</t>
+  </si>
+  <si>
+    <t>nothing special , regular day</t>
+  </si>
+  <si>
+    <t>August/September</t>
   </si>
 </sst>
 </file>
@@ -981,7 +984,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="G3" s="20"/>
     </row>
@@ -1008,7 +1011,7 @@
         <v>35</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>36</v>
@@ -1130,13 +1133,13 @@
         <v>48</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M7" s="16" t="s">
         <v>50</v>
       </c>
       <c r="N7" s="17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1173,16 +1176,16 @@
         <v>195</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M8" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N8" s="17" t="s">
         <v>59</v>
-      </c>
-      <c r="N8" s="17" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -1219,16 +1222,16 @@
         <v>240</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L9" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N9" s="17" t="s">
         <v>61</v>
-      </c>
-      <c r="M9" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="N9" s="17" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -1274,7 +1277,7 @@
         <v>50</v>
       </c>
       <c r="N10" s="17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
@@ -1320,7 +1323,7 @@
         <v>50</v>
       </c>
       <c r="N11" s="17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -1366,7 +1369,7 @@
         <v>50</v>
       </c>
       <c r="N12" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1403,7 +1406,7 @@
         <v>100</v>
       </c>
       <c r="K13" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L13" s="16" t="s">
         <v>49</v>
@@ -1412,7 +1415,7 @@
         <v>50</v>
       </c>
       <c r="N13" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
@@ -1449,16 +1452,16 @@
         <v>0</v>
       </c>
       <c r="K14" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L14" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="L14" s="16" t="s">
+      <c r="M14" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="M14" s="16" t="s">
+      <c r="N14" s="17" t="s">
         <v>68</v>
-      </c>
-      <c r="N14" s="17" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -1498,13 +1501,13 @@
         <v>48</v>
       </c>
       <c r="L15" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M15" s="16" t="s">
         <v>50</v>
       </c>
       <c r="N15" s="17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1550,7 +1553,7 @@
         <v>50</v>
       </c>
       <c r="N16" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
@@ -1587,7 +1590,7 @@
         <v>30</v>
       </c>
       <c r="K17" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L17" s="16" t="s">
         <v>49</v>
@@ -1596,7 +1599,7 @@
         <v>50</v>
       </c>
       <c r="N17" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
@@ -1633,16 +1636,16 @@
         <v>40</v>
       </c>
       <c r="K18" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L18" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N18" s="17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1679,16 +1682,16 @@
         <v>40</v>
       </c>
       <c r="K19" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L19" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="L19" s="16" t="s">
+      <c r="M19" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="M19" s="16" t="s">
-        <v>68</v>
-      </c>
       <c r="N19" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
@@ -1734,7 +1737,7 @@
         <v>50</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
@@ -1780,30 +1783,54 @@
         <v>50</v>
       </c>
       <c r="N21" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B22" s="14">
+        <v>360</v>
+      </c>
+      <c r="C22" s="14">
+        <v>30</v>
+      </c>
+      <c r="D22" s="14">
+        <v>180</v>
+      </c>
+      <c r="E22" s="14">
+        <v>30</v>
+      </c>
+      <c r="F22" s="14">
+        <v>360</v>
+      </c>
+      <c r="G22" s="14">
+        <v>5</v>
+      </c>
+      <c r="H22" s="14">
+        <v>480</v>
+      </c>
+      <c r="I22" s="15">
+        <f t="shared" si="0"/>
+        <v>1440</v>
+      </c>
+      <c r="J22" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N22" s="17" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="13"/>

</xml_diff>

<commit_message>
New month Second Commit
</commit_message>
<xml_diff>
--- a/12620583.xlsx
+++ b/12620583.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VITHOBA_12620583\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E784FF0E-2A68-471B-BED4-293D73D3B500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34ABE24A-6160-4957-B2F2-7E7EC1D16594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="116">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -367,6 +367,24 @@
   <si>
     <t>Today I drive a tractor after many days</t>
   </si>
+  <si>
+    <t>normal day but I work in farm</t>
+  </si>
+  <si>
+    <t>good filings just because I meet my sister</t>
+  </si>
+  <si>
+    <t>regular day but at home energy is high</t>
+  </si>
+  <si>
+    <t>same like yesterday</t>
+  </si>
+  <si>
+    <t>I get my bike back and enjoy the ride</t>
+  </si>
+  <si>
+    <t>today I went to taluka and enjoy with friends</t>
+  </si>
 </sst>
 </file>
 
@@ -545,9 +563,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1043,74 +1061,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="20">
         <v>12620583</v>
       </c>
-      <c r="G2" s="19"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
       <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="20"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
     </row>
     <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -11022,74 +11040,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="20">
         <v>12620583</v>
       </c>
-      <c r="G2" s="19"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
       <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="20"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
     </row>
     <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -11227,53 +11245,97 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
         <v>46297</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="15" t="str">
+      <c r="B8" s="14">
+        <v>420</v>
+      </c>
+      <c r="C8" s="14">
+        <v>30</v>
+      </c>
+      <c r="D8" s="14">
+        <v>0</v>
+      </c>
+      <c r="E8" s="14">
+        <v>0</v>
+      </c>
+      <c r="F8" s="14">
+        <v>0</v>
+      </c>
+      <c r="G8" s="14">
+        <v>0</v>
+      </c>
+      <c r="H8" s="14">
+        <v>950</v>
+      </c>
+      <c r="I8" s="15">
         <f t="shared" ref="I8:I58" si="2">IF(SUM(B8:F8,H8)=0,"",SUM(B8:F8,H8))</f>
-        <v/>
-      </c>
-      <c r="J8" s="15" t="str">
+        <v>1400</v>
+      </c>
+      <c r="J8" s="15">
         <f t="shared" ref="J8:J58" si="3">IF(I8="","",1440-I8)</f>
-        <v/>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="17"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
         <v>46298</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+      <c r="B9" s="14">
+        <v>420</v>
+      </c>
+      <c r="C9" s="14">
+        <v>0</v>
+      </c>
+      <c r="D9" s="14">
+        <v>0</v>
+      </c>
+      <c r="E9" s="14">
+        <v>0</v>
+      </c>
+      <c r="F9" s="14">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14">
+        <v>0</v>
+      </c>
+      <c r="H9" s="14">
+        <v>1000</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>1420</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
+        <v>20</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="10" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="13">
@@ -11322,136 +11384,280 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+      <c r="A11" s="13">
+        <v>46300</v>
+      </c>
+      <c r="B11" s="14">
+        <v>360</v>
+      </c>
+      <c r="C11" s="14">
+        <v>60</v>
+      </c>
+      <c r="D11" s="14">
+        <v>0</v>
+      </c>
+      <c r="E11" s="14">
+        <v>0</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14">
+        <v>0</v>
+      </c>
+      <c r="H11" s="14">
+        <v>1000</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>1420</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="17"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+        <v>20</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
+        <v>46301</v>
+      </c>
+      <c r="B12" s="14">
+        <v>360</v>
+      </c>
+      <c r="C12" s="14">
+        <v>60</v>
+      </c>
+      <c r="D12" s="14">
+        <v>0</v>
+      </c>
+      <c r="E12" s="14">
+        <v>0</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14">
+        <v>1000</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>1420</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+        <v>20</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="13">
+        <v>46302</v>
+      </c>
+      <c r="B13" s="14">
+        <v>420</v>
+      </c>
+      <c r="C13" s="14">
+        <v>60</v>
+      </c>
+      <c r="D13" s="14">
+        <v>0</v>
+      </c>
+      <c r="E13" s="14">
+        <v>0</v>
+      </c>
+      <c r="F13" s="14">
+        <v>0</v>
+      </c>
+      <c r="G13" s="14">
+        <v>0</v>
+      </c>
+      <c r="H13" s="14">
+        <v>950</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>1430</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
+        <v>10</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="A14" s="13">
+        <v>46303</v>
+      </c>
+      <c r="B14" s="14">
+        <v>420</v>
+      </c>
+      <c r="C14" s="14">
+        <v>40</v>
+      </c>
+      <c r="D14" s="14">
+        <v>0</v>
+      </c>
+      <c r="E14" s="14">
+        <v>0</v>
+      </c>
+      <c r="F14" s="14">
+        <v>0</v>
+      </c>
+      <c r="G14" s="14">
+        <v>0</v>
+      </c>
+      <c r="H14" s="14">
+        <v>950</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>1410</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>30</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+      <c r="A15" s="13">
+        <v>46304</v>
+      </c>
+      <c r="B15" s="14">
+        <v>420</v>
+      </c>
+      <c r="C15" s="14">
+        <v>30</v>
+      </c>
+      <c r="D15" s="14">
+        <v>0</v>
+      </c>
+      <c r="E15" s="14">
+        <v>0</v>
+      </c>
+      <c r="F15" s="14">
+        <v>0</v>
+      </c>
+      <c r="G15" s="14">
+        <v>0</v>
+      </c>
+      <c r="H15" s="14">
+        <v>950</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>1400</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="17"/>
+        <v>40</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+      <c r="A16" s="13">
+        <v>46305</v>
+      </c>
+      <c r="B16" s="14">
+        <v>420</v>
+      </c>
+      <c r="C16" s="14">
+        <v>30</v>
+      </c>
+      <c r="D16" s="14">
+        <v>0</v>
+      </c>
+      <c r="E16" s="14">
+        <v>0</v>
+      </c>
+      <c r="F16" s="14">
+        <v>0</v>
+      </c>
+      <c r="G16" s="14">
+        <v>0</v>
+      </c>
+      <c r="H16" s="14">
+        <v>950</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>1400</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="17"/>
+        <v>40</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="13"/>

</xml_diff>

<commit_message>
after break commit 1
</commit_message>
<xml_diff>
--- a/12620583.xlsx
+++ b/12620583.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VITHOBA_12620583\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34ABE24A-6160-4957-B2F2-7E7EC1D16594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5023C9E8-23E0-44AE-9DD5-19A8731495E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="124">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -384,6 +384,30 @@
   </si>
   <si>
     <t>today I went to taluka and enjoy with friends</t>
+  </si>
+  <si>
+    <t>Back to college and started study for Mid Term</t>
+  </si>
+  <si>
+    <t xml:space="preserve">today Mid term start and sub was networking medium level  harder  </t>
+  </si>
+  <si>
+    <t>today was cpp exam and it's very simple exam I ever give in any college</t>
+  </si>
+  <si>
+    <t>today was database exam and it's simple but having some issue with  some querys</t>
+  </si>
+  <si>
+    <t>today was holiday day and watch movie more than study</t>
+  </si>
+  <si>
+    <t>today was aptii exam it's very difficult and I didn't attend all questions [ just because I didn't understand syllabus ].</t>
+  </si>
+  <si>
+    <t>today was communication exam I give my best and I think the exam was very simple from my side I mark all questions write but let's see what happens…</t>
+  </si>
+  <si>
+    <t>today is holiday and I started my personal study and also I think to continue my diary writing from today itself..</t>
   </si>
 </sst>
 </file>
@@ -11659,181 +11683,373 @@
         <v>113</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+    <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="13">
+        <v>46306</v>
+      </c>
+      <c r="B17" s="14">
+        <v>540</v>
+      </c>
+      <c r="C17" s="14">
+        <v>0</v>
+      </c>
+      <c r="D17" s="14">
+        <v>300</v>
+      </c>
+      <c r="E17" s="14">
+        <v>120</v>
+      </c>
+      <c r="F17" s="14">
+        <v>0</v>
+      </c>
+      <c r="G17" s="14">
+        <v>0</v>
+      </c>
+      <c r="H17" s="14">
+        <v>480</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+        <v>0</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="13">
+        <v>46307</v>
+      </c>
+      <c r="B18" s="14">
+        <v>360</v>
+      </c>
+      <c r="C18" s="14">
+        <v>30</v>
+      </c>
+      <c r="D18" s="14">
+        <v>120</v>
+      </c>
+      <c r="E18" s="14">
+        <v>0</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0</v>
+      </c>
+      <c r="H18" s="14">
+        <v>800</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>1310</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+        <v>130</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="13">
+        <v>46308</v>
+      </c>
+      <c r="B19" s="14">
+        <v>420</v>
+      </c>
+      <c r="C19" s="14">
+        <v>30</v>
+      </c>
+      <c r="D19" s="14">
+        <v>360</v>
+      </c>
+      <c r="E19" s="14">
+        <v>120</v>
+      </c>
+      <c r="F19" s="14">
+        <v>0</v>
+      </c>
+      <c r="G19" s="14">
+        <v>0</v>
+      </c>
+      <c r="H19" s="14">
+        <v>500</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>1430</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+        <v>10</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="13">
+        <v>46309</v>
+      </c>
+      <c r="B20" s="14">
+        <v>420</v>
+      </c>
+      <c r="C20" s="14">
+        <v>30</v>
+      </c>
+      <c r="D20" s="14">
+        <v>360</v>
+      </c>
+      <c r="E20" s="14">
+        <v>120</v>
+      </c>
+      <c r="F20" s="14">
+        <v>0</v>
+      </c>
+      <c r="G20" s="14">
+        <v>0</v>
+      </c>
+      <c r="H20" s="14">
+        <v>480</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>1410</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+        <v>30</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="13">
+        <v>46310</v>
+      </c>
+      <c r="B21" s="14">
+        <v>600</v>
+      </c>
+      <c r="C21" s="14">
+        <v>30</v>
+      </c>
+      <c r="D21" s="14">
+        <v>180</v>
+      </c>
+      <c r="E21" s="14">
+        <v>0</v>
+      </c>
+      <c r="F21" s="14">
+        <v>0</v>
+      </c>
+      <c r="G21" s="14">
+        <v>0</v>
+      </c>
+      <c r="H21" s="14">
+        <v>600</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>1410</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+        <v>30</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
+        <v>46311</v>
+      </c>
+      <c r="B22" s="14">
+        <v>420</v>
+      </c>
+      <c r="C22" s="14">
+        <v>30</v>
+      </c>
+      <c r="D22" s="14">
+        <v>360</v>
+      </c>
+      <c r="E22" s="14">
+        <v>0</v>
+      </c>
+      <c r="F22" s="14">
+        <v>0</v>
+      </c>
+      <c r="G22" s="14">
+        <v>0</v>
+      </c>
+      <c r="H22" s="14">
+        <v>600</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>1410</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+        <v>30</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A23" s="13">
+        <v>46312</v>
+      </c>
+      <c r="B23" s="14">
+        <v>420</v>
+      </c>
+      <c r="C23" s="14">
+        <v>30</v>
+      </c>
+      <c r="D23" s="14">
+        <v>360</v>
+      </c>
+      <c r="E23" s="14">
+        <v>0</v>
+      </c>
+      <c r="F23" s="14">
+        <v>0</v>
+      </c>
+      <c r="G23" s="14">
+        <v>0</v>
+      </c>
+      <c r="H23" s="14">
+        <v>600</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1410</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+        <v>30</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="13">
+        <v>46313</v>
+      </c>
+      <c r="B24" s="14">
+        <v>180</v>
+      </c>
+      <c r="C24" s="14">
+        <v>60</v>
+      </c>
+      <c r="D24" s="14">
+        <v>560</v>
+      </c>
+      <c r="E24" s="14">
+        <v>120</v>
+      </c>
+      <c r="F24" s="14">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14">
+        <v>0</v>
+      </c>
+      <c r="H24" s="14">
+        <v>500</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>1420</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
+        <v>20</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="13"/>

</xml_diff>